<commit_message>
Matching work to 50%
</commit_message>
<xml_diff>
--- a/Section_Notes.xlsx
+++ b/Section_Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/quinnmackay/Documents/GitHub/BICC_Holocene_LayerCount/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC55CACF-B0CF-9D4A-A13D-8C443C67CBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C482CB0F-B754-0440-B7AE-195B8417AC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30240" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30240" yWindow="660" windowWidth="30240" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="97">
   <si>
     <t>EDML m</t>
   </si>
@@ -243,6 +243,87 @@
   </si>
   <si>
     <t>Cut 214.3, 215.7, 217.7, 219.4, 221.75, 226.6, 227.8, 227.45, 214.25</t>
+  </si>
+  <si>
+    <t>Added one to EDML at 231.55, removed one from WDC: 718.5</t>
+  </si>
+  <si>
+    <t>From EDML: Dropped 236.25, uncertain 240.75, double peak at 238.3 and 238.35 and 237.4 and 235.6.</t>
+  </si>
+  <si>
+    <t>Kept 0.5 at 245.4, removed rest. Reduced blank spot around 242.7 by 1. Removed double peak at 244.4, peak at 246.25</t>
+  </si>
+  <si>
+    <t>Added uncertainties at 248.9, 250.25 and 249.55. I think one more but forgot which one. Removed from WD at 772.1 and 784.1 and 779.25</t>
+  </si>
+  <si>
+    <t>Added uncertainty at 254.52 and 255.95, SUPER uncertain at 255.55</t>
+  </si>
+  <si>
+    <t>Dropped 259.2, 265.5, 260.05. All were uncertain</t>
+  </si>
+  <si>
+    <t>Dropped 268.3, 267.605, 266.3, 266.405</t>
+  </si>
+  <si>
+    <t>Added uncertain at 270.3</t>
+  </si>
+  <si>
+    <t>Kept 271.4 (although very weak but wide spacing), dropped all other 0.5. Dropped 271.35. Moved the one to the left a bit to the right.</t>
+  </si>
+  <si>
+    <t>Dropped all 0.5 and 274.1</t>
+  </si>
+  <si>
+    <t>Dropped 275.85, 275.67, 275.02, 248.85</t>
+  </si>
+  <si>
+    <t>Dropped 278.45. Kept 0.5 at: 276.65, 278.4, 280.2, 280.9, 281.85, 282.8, 283.2, 235.75, 235.85, 284.45</t>
+  </si>
+  <si>
+    <t>Added uncertain EDML at 258.92</t>
+  </si>
+  <si>
+    <t>Dropped uncertain at 287.8 and 286.6</t>
+  </si>
+  <si>
+    <t>Added uncertain at 290.75</t>
+  </si>
+  <si>
+    <t>Added uncertain at 293.7 and 295.6</t>
+  </si>
+  <si>
+    <t>dropped 296.95, 301.95, 302.78, 305.75, 309.9, 308.4, 308.55, 308.15, 306.5, 299.4</t>
+  </si>
+  <si>
+    <t>Cut uncertain 311.8</t>
+  </si>
+  <si>
+    <t>Cut uncertain at 314.5. This is a really hard one (tiepoint problem?), Added new weak WDC tiepoint at about 987.2. Took two at 315.8 and made one. Removed 315.3</t>
+  </si>
+  <si>
+    <t>Dropped all uncertains except 316.65</t>
+  </si>
+  <si>
+    <t>Dropped uncertain at 319.7</t>
+  </si>
+  <si>
+    <t>Dropped uncertain at 322.05, 321.75, 322.2. Dropped full at 321.25</t>
+  </si>
+  <si>
+    <t>Dropped uncertain at 322.83, dropped full at 322.65</t>
+  </si>
+  <si>
+    <t>Removed all uncertain from EDML, added one to WDC at 1018.5 (uncertain)</t>
+  </si>
+  <si>
+    <t>Dropped full at 325.75, moved uncertain right by it. Dropped 327.25, 327.8, 328.2, 328.6, 329.05</t>
+  </si>
+  <si>
+    <t>Dropped uncertain at 329.6, 333.4, 334.45, 332.6, 333.45 (moved full just to the right of it to the left).</t>
+  </si>
+  <si>
+    <t>Another really hard one. Dropped uncertain at 337.7, dropped full at 337.85, 336.55. Added to WDC at 1057.9 and 1058.15.</t>
   </si>
 </sst>
 </file>
@@ -271,12 +352,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -317,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -326,6 +413,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1594,7 +1682,7 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38">
+      <c r="A38" s="4">
         <v>37</v>
       </c>
       <c r="B38">
@@ -1615,9 +1703,12 @@
       <c r="G38">
         <v>-2.8848171641493541</v>
       </c>
+      <c r="H38" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39">
+      <c r="A39" s="4">
         <v>38</v>
       </c>
       <c r="B39">
@@ -1638,9 +1729,12 @@
       <c r="G39">
         <v>7.4451299948377709</v>
       </c>
+      <c r="H39" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40">
+      <c r="A40" s="4">
         <v>39</v>
       </c>
       <c r="B40">
@@ -1661,9 +1755,12 @@
       <c r="G40">
         <v>11.898560375443139</v>
       </c>
+      <c r="H40" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41">
+      <c r="A41" s="4">
         <v>40</v>
       </c>
       <c r="B41">
@@ -1684,9 +1781,12 @@
       <c r="G41">
         <v>-6.6266730271750021</v>
       </c>
+      <c r="H41" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42">
+      <c r="A42" s="4">
         <v>41</v>
       </c>
       <c r="B42">
@@ -1707,9 +1807,12 @@
       <c r="G42">
         <v>-3.1819961220908231</v>
       </c>
+      <c r="H42" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43">
+      <c r="A43" s="4">
         <v>42</v>
       </c>
       <c r="B43">
@@ -1730,9 +1833,12 @@
       <c r="G43">
         <v>0.3511194676143532</v>
       </c>
+      <c r="H43" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44">
+      <c r="A44" s="4">
         <v>43</v>
       </c>
       <c r="B44">
@@ -1753,9 +1859,12 @@
       <c r="G44">
         <v>2.2364046166708249</v>
       </c>
+      <c r="H44" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45">
+      <c r="A45" s="4">
         <v>44</v>
       </c>
       <c r="B45">
@@ -1776,9 +1885,12 @@
       <c r="G45">
         <v>4.4649839155513291</v>
       </c>
+      <c r="H45" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46">
+      <c r="A46" s="4">
         <v>45</v>
       </c>
       <c r="B46">
@@ -1799,9 +1911,12 @@
       <c r="G46">
         <v>-0.41843244660685741</v>
       </c>
+      <c r="H46" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47">
+      <c r="A47" s="4">
         <v>46</v>
       </c>
       <c r="B47">
@@ -1822,9 +1937,12 @@
       <c r="G47">
         <v>4.1499836902012248</v>
       </c>
+      <c r="H47" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48">
+      <c r="A48" s="4">
         <v>47</v>
       </c>
       <c r="B48">
@@ -1845,9 +1963,12 @@
       <c r="G48">
         <v>4.5589685278023353</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49">
+      <c r="H48" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="4">
         <v>48</v>
       </c>
       <c r="B49">
@@ -1868,9 +1989,12 @@
       <c r="G49">
         <v>4.3700463696090992</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50">
+      <c r="H49" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="4">
         <v>49</v>
       </c>
       <c r="B50">
@@ -1891,9 +2015,12 @@
       <c r="G50">
         <v>13.967906952668731</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51">
+      <c r="H50" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="4">
         <v>50</v>
       </c>
       <c r="B51">
@@ -1914,9 +2041,12 @@
       <c r="G51">
         <v>-1.023754637490583</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52">
+      <c r="H51" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="4">
         <v>51</v>
       </c>
       <c r="B52">
@@ -1937,9 +2067,12 @@
       <c r="G52">
         <v>2.5274697908371309</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A53">
+      <c r="H52" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="4">
         <v>52</v>
       </c>
       <c r="B53">
@@ -1960,9 +2093,12 @@
       <c r="G53">
         <v>-0.52176357120879402</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54">
+      <c r="H53" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="4">
         <v>53</v>
       </c>
       <c r="B54">
@@ -1983,9 +2119,12 @@
       <c r="G54">
         <v>-1.872669285487973</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55">
+      <c r="H54" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="4">
         <v>54</v>
       </c>
       <c r="B55">
@@ -2006,9 +2145,12 @@
       <c r="G55">
         <v>9.2227808982274837</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56">
+      <c r="H55" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="4">
         <v>55</v>
       </c>
       <c r="B56">
@@ -2029,9 +2171,12 @@
       <c r="G56">
         <v>1.6637510585069319</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57">
+      <c r="H56" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="4">
         <v>56</v>
       </c>
       <c r="B57">
@@ -2052,9 +2197,12 @@
       <c r="G57">
         <v>3.7730450430153719</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A58">
+      <c r="H57" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="4">
         <v>57</v>
       </c>
       <c r="B58">
@@ -2075,9 +2223,12 @@
       <c r="G58">
         <v>3.4410789075500361</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A59">
+      <c r="H58" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="4">
         <v>58</v>
       </c>
       <c r="B59">
@@ -2098,9 +2249,12 @@
       <c r="G59">
         <v>1.346108227573495</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A60">
+      <c r="H59" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="4">
         <v>59</v>
       </c>
       <c r="B60">
@@ -2121,9 +2275,12 @@
       <c r="G60">
         <v>3.556648906223018</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61">
+      <c r="H60" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="4">
         <v>60</v>
       </c>
       <c r="B61">
@@ -2144,9 +2301,12 @@
       <c r="G61">
         <v>2.381604067152693</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A62">
+      <c r="H61" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="4">
         <v>61</v>
       </c>
       <c r="B62">
@@ -2167,9 +2327,12 @@
       <c r="G62">
         <v>4.8965199730910172</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A63">
+      <c r="H62" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="4">
         <v>62</v>
       </c>
       <c r="B63">
@@ -2190,9 +2353,12 @@
       <c r="G63">
         <v>6.2015099644941074</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A64">
+      <c r="H63" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" s="4">
         <v>63</v>
       </c>
       <c r="B64">
@@ -2213,9 +2379,12 @@
       <c r="G64">
         <v>3.4653823279968492</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65">
+      <c r="H64" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" s="4">
         <v>64</v>
       </c>
       <c r="B65">
@@ -2236,8 +2405,11 @@
       <c r="G65">
         <v>3.9983731130832889</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H65" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2260,7 +2432,7 @@
         <v>22.665157008064849</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2283,7 +2455,7 @@
         <v>12.350105362253091</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2306,7 +2478,7 @@
         <v>6.459456358135867</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2329,7 +2501,7 @@
         <v>3.2318920868747232</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2352,7 +2524,7 @@
         <v>7.6392241042103706</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2375,7 +2547,7 @@
         <v>3.4019300691097669</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2398,7 +2570,7 @@
         <v>-6.3959376855564187E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2421,7 +2593,7 @@
         <v>2.9747550431557102</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2444,7 +2616,7 @@
         <v>7.7548566821724307</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2467,7 +2639,7 @@
         <v>0.30416190951928002</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2490,7 +2662,7 @@
         <v>0.78476532274635247</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2513,7 +2685,7 @@
         <v>1.3971929666286089</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2536,7 +2708,7 @@
         <v>1.6020007209972389</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2559,7 +2731,7 @@
         <v>9.4735812131511921</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>

</xml_diff>